<commit_message>
made final input, dashboard and feedback changes in agent 1
</commit_message>
<xml_diff>
--- a/agent-3/inputs/search_request.xlsx
+++ b/agent-3/inputs/search_request.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ananya.Mehta\OneDrive - Parkar\Desktop\redpine-ai\agent-3\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFBB71EE-F661-4447-B2B7-3E883CBC9D3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F628A907-8111-4A14-8A56-87153C20E40C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="740" windowWidth="19180" windowHeight="10060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Geography</t>
   </si>
@@ -46,9 +46,6 @@
   </si>
   <si>
     <t>Florida</t>
-  </si>
-  <si>
-    <t>Manufacturing</t>
   </si>
   <si>
     <t>$10M-$50M</t>
@@ -427,30 +424,28 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="2"/>
+      <c r="C2" s="2" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
       </c>
       <c r="D2" s="2">
         <v>20</v>
       </c>
       <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="G2" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">

</xml_diff>